<commit_message>
some changes in backend & frontend
</commit_message>
<xml_diff>
--- a/project-management/SmartKhata_Project_Management.xlsx
+++ b/project-management/SmartKhata_Project_Management.xlsx
@@ -183,27 +183,27 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>64</t>
+          <t>67</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>79</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>74</t>
+          <t>77</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>71</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -662,12 +662,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Suppliers Legacy</t>
+          <t>Shopping Products</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>/api/suppliers</t>
+          <t>/api/shopping/products</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -677,34 +677,34 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Manual pending</t>
+          <t>Build passed; manual pending</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>82</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Shopping Products</t>
+          <t>Shopping Orders</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>/api/shopping/products</t>
+          <t>/api/shopping/orders</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>GET/POST/PUT/DELETE</t>
+          <t>GET/POST</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -726,17 +726,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Shopping Orders</t>
+          <t>Shopping Order Status</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>/api/shopping/orders</t>
+          <t>/api/shopping/orders/:id/status</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>GET/POST</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -751,24 +751,24 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>82</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Shopping Order Status</t>
+          <t>Staff Summary</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>/api/shopping/orders/:id/status</t>
+          <t>/api/staff/summary</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -783,24 +783,24 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>88</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Staff Summary</t>
+          <t>Staff CRUD</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>/api/staff/summary</t>
+          <t>/api/staff</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>GET/POST/PUT/DELETE</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -815,24 +815,24 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>86</t>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Staff CRUD</t>
+          <t>Staff History</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>/api/staff</t>
+          <t>/api/staff/:id/history</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>GET/POST/PUT/DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -847,51 +847,51 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>82</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Staff History</t>
+          <t>Staff Attendance</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>/api/staff/:id/history</t>
+          <t>/api/staff/:id/attendance</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Service ready</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Build passed; UI pending</t>
+          <t>Build passed; manual pending</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>82</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Staff Attendance</t>
+          <t>Staff Salary Payments</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>/api/staff/:id/attendance</t>
+          <t>/api/staff/:id/salary-payments</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -901,7 +901,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Service ready</t>
+          <t>Backend ready; frontend static</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -911,19 +911,19 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>72</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Staff Salary Payments</t>
+          <t>Staff Advances</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>/api/staff/:id/salary-payments</t>
+          <t>/api/staff/:id/advances</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -933,7 +933,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Service ready</t>
+          <t>Backend ready; frontend static</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -943,56 +943,56 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>72</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Staff Advances</t>
+          <t>Inventory Products</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>/api/staff/:id/advances</t>
+          <t>/api/inventory/products</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET/POST/PUT/DELETE</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Service ready</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Build passed; UI pending</t>
+          <t>Build passed; manual pending</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>86</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Inventory Products</t>
+          <t>Inventory Stock Update</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>/api/inventory/products</t>
+          <t>/api/inventory/products/:id/stock</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>GET/POST/PUT/DELETE</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1014,17 +1014,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Inventory Stock Update</t>
+          <t>Inventory History</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>/api/inventory/products/:id/stock</t>
+          <t>/api/inventory/history</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1046,12 +1046,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Inventory History</t>
+          <t>Inventory Summary</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>/api/inventory/history</t>
+          <t>/api/inventory/summary</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1078,17 +1078,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Inventory Summary</t>
+          <t>Collections Compatibility</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>/api/inventory/summary</t>
+          <t>/api/collections/*</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>GET/POST/PUT/PATCH/DELETE</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1103,76 +1103,44 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>86</t>
+          <t>82</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Collections Compatibility</t>
+          <t>Transactions</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>/api/collections/*</t>
+          <t>/api/transactions</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>GET/POST/PUT/PATCH/DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Build passed; manual pending</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>82</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Transactions</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>/api/transactions</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
           <t>0</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F29"/>
+  <autoFilter ref="A1:F28"/>
 </worksheet>
 </file>
 
@@ -1419,7 +1387,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Staff attendance/salary/advance APIs exist but frontend forms/history are not implemented</t>
+          <t>Staff salary/advance/document/report sections are visible but not fully wired to real backend data</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1515,7 +1483,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Staff frontend includes employee_id/email/department fields but backend currently persists only name/mobile/role/salary/date/status/address/note</t>
+          <t>Staff form field persistence mismatch resolved for staff_id/email/department</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1530,12 +1498,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -2031,7 +1999,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Passed on 2026-07-01</t>
+          <t>Passed on 2026-07-01 after latest Staff/Shopping updates</t>
         </is>
       </c>
     </row>
@@ -2127,7 +2095,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Passed on 2026-07-01</t>
+          <t>Passed on 2026-07-01 after latest Staff/Shopping updates</t>
         </is>
       </c>
     </row>
@@ -2423,7 +2391,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Staff advanced workflows have backend APIs but frontend forms/history are pending</t>
+          <t>Staff salary, advance, document and report sections are partly static</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2438,7 +2406,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Add attendance, salary, advance and history UI sections</t>
+          <t>Wire sections to existing APIs or mark as preview states</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -2546,17 +2514,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Data Model</t>
+          <t>Resolved</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Staff form fields employee_id/email/department are not persisted by backend schema</t>
+          <t>Staff form fields staff_id/email/department are now persisted by backend schema</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -2566,12 +2534,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Add backend columns or remove frontend fields</t>
+          <t>Continue manual DB verification</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -2625,12 +2593,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>68</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -2640,7 +2608,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Dashboard, Customers, Inventory, Shopping, Orders, Staff, Supplier split and project management updates progressed through 2026-07-01</t>
+          <t>Dashboard, Customers, Inventory, Shopping, Orders, Staff HRMS, Supplier split and project management updates progressed through 2026-07-01</t>
         </is>
       </c>
     </row>
@@ -2719,12 +2687,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Project baseline Excel; Inventory replacement; Dashboard live aggregation; Customers page upgrade; Shopping UI/order board upgrade; standalone Orders page; Staff core module; supplier/customer credit API split; frontend build verification on 2026-07-01</t>
+          <t>Project baseline Excel; Inventory replacement; Dashboard live aggregation; Customers page upgrade; Shopping catalog cleanup; standalone Orders page; Staff HRMS expansion; staff_id/email/department backend persistence; supplier/customer credit API split; frontend build verification on 2026-07-01</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Staff advanced UI; customer product entry edit/delete UI check; dashboard fallback cleanup; manual QA</t>
+          <t>Staff salary/advance/document/report real-data wiring; dashboard fallback cleanup; manual QA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2734,32 +2702,32 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>No automated tests; hardcoded DB config; reports/settings/transactions placeholders; manual MySQL QA pending; Staff form/backend field mismatch</t>
+          <t>No automated tests; hardcoded DB config; reports/settings/transactions placeholders; manual MySQL QA pending</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Orders placeholder resolved; Credit module split; Staff module added; shopping service moved to services; inventory service moved to services</t>
+          <t>Staff field persistence mismatch closed; Shopping separated from Orders; latest frontend build passed</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>68</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>64</t>
+          <t>67</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Transactions API/page, Staff advanced UI alignment, Reports foundation</t>
+          <t>Transactions API/page, Staff real-data wiring, Reports foundation</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -2854,17 +2822,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Orders implemented; Staff module added; supplier/customer credit architecture split; frontend build passed on 2026-07-01</t>
+          <t>Orders implemented; Staff HRMS expanded; staff persistence fixed; supplier/customer credit architecture split; latest frontend build passed on 2026-07-01</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Project management baseline, Inventory module, Dashboard integration, Customer ledger upgrade, Shopping UX, Orders page, Staff core CRUD, Supplier purchase split</t>
+          <t>Project management baseline, Inventory module, Dashboard integration, Customer ledger upgrade, Shopping catalog, Orders page, Staff CRUD/attendance UI, Supplier purchase split</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Transactions, Reports, Settings, Staff advanced frontend, automated tests, deployment/security hardening</t>
+          <t>Transactions, Reports, Settings, Staff salary/advance/document real-data wiring, automated tests, deployment/security hardening</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -2879,7 +2847,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>No automated tests, hardcoded DB password, dashboard fallback data, Staff field persistence mismatch</t>
+          <t>No automated tests, hardcoded DB password, dashboard fallback data, static staff subsections</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -2889,7 +2857,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>64</t>
+          <t>67</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -2996,62 +2964,62 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>79</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>74</t>
+          <t>77</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>71</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Needs hardening</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Vite production build passed; no performance audit</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Reports/settings/transactions incomplete; no automated tests; hardcoded DB config; dashboard fallbacks; Staff salary/advance/document real-data wiring pending; manual DB QA pending</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
           <t>68</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>75</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Needs hardening</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Vite production build passed; no performance audit</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Reports/settings/transactions incomplete; no automated tests; hardcoded DB config; dashboard fallbacks; Staff advanced UI pending; Staff field persistence mismatch; manual DB QA pending</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>65</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -3447,109 +3415,109 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Adesh/Dev Team</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>SmartKhata</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Sprint 1</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Customer Ledger</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Customer detail and product entry</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>SK-005</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Enhanced customer page with summary cards, selected customer panel, product entry and unified history</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Build Passed</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Needs manual CRUD/history verification with MySQL</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Adesh/Dev Team</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>SmartKhata</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Analytics</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Live dashboard aggregation</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>SK-001</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Connected dashboard with customers, credits, payments, orders and inventory data</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>No Change</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>Integrated</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Build Passed</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>75</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>Fallback mock values still present</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>2026-06-24</t>
-        </is>
-      </c>
       <c r="V4" t="inlineStr">
         <is>
           <t>2026-06-25</t>
@@ -3557,14 +3525,14 @@
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>Production build verified</t>
+          <t>Customer history includes payments, product entries and shopping orders</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -3579,32 +3547,32 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
+          <t>Sprint 2</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Customers</t>
+          <t>Orders</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Customer Ledger</t>
+          <t>Standalone Orders</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Customer detail and product entry</t>
+          <t>Order management screen</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>SK-005</t>
+          <t>SK-W2-002</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Enhanced customer page with summary cards, selected customer panel, product entry and unified history</t>
+          <t>Built full Orders page with summary cards, order search/filter, status updates, product list and refresh</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -3619,12 +3587,12 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>No Change</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -3644,7 +3612,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -3659,29 +3627,29 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>Needs manual CRUD/history verification with MySQL</t>
+          <t>Manual DB order status testing pending</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>Customer history includes payments, product entries and shopping orders</t>
+          <t>Orders page no longer placeholder</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -3696,32 +3664,32 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
+          <t>Sprint 2</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Shopping</t>
+          <t>Staff</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Shopping Orders</t>
+          <t>Staff Management</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Product catalog and order board</t>
+          <t>Staff CRUD and staff finance APIs</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>SK-006</t>
+          <t>SK-W2-006</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Improved shopping page UI, product CRUD, order filters/status and product preview modal</t>
+          <t>Added Staff module with frontend page, sidebar route, backend staff CRUD, summary, attendance, salary payment and advance APIs</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -3756,49 +3724,49 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>78</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>QA</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>Manual order flow testing pending</t>
+          <t>Attendance/salary/advance frontend screens pending</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>Orders functional inside Shopping page</t>
+          <t>Core staff CRUD UI done; advanced staff APIs exist</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -3818,27 +3786,27 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Orders</t>
+          <t>Supplier/Credit</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Standalone Orders</t>
+          <t>Architecture Split</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Order management screen</t>
+          <t>Supplier purchases and customer credits</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>SK-W2-002</t>
+          <t>SK-W2-007</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Built full Orders page with summary cards, order search/filter, status updates, product list and refresh</t>
+          <t>Split old credit module into supplier-purchases and customer-credits APIs/services; updated supplier route to /supplier</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -3853,12 +3821,12 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>No Change</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Integrated</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -3873,17 +3841,17 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>82</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -3893,22 +3861,22 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>Manual DB order status testing pending</t>
+          <t>Manual old route regression pending</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>Orders page no longer placeholder</t>
+          <t>Old Credit.jsx/Credit.css and creditRoutes removed</t>
         </is>
       </c>
     </row>
@@ -3940,22 +3908,22 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Staff Management</t>
+          <t>HRMS Expansion</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Staff CRUD and staff finance APIs</t>
+          <t>Staff profile, attendance and staff dashboard</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>SK-W2-006</t>
+          <t>SK-W2-009</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Added Staff module with frontend page, sidebar route, backend staff CRUD, summary, attendance, salary payment and advance APIs</t>
+          <t>Expanded Staff page with HRMS navigation, staff filters/sort, persisted staff_id/email/department, attendance entry/history, salary/advance/leave/performance/document/report sections</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -3975,7 +3943,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Integrated</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -3990,27 +3958,27 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>88</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>QA</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>Attendance/salary/advance frontend screens pending</t>
+          <t>Salary/advance/document/report sections still partly static</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -4025,7 +3993,7 @@
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>Core staff CRUD UI done; advanced staff APIs exist</t>
+          <t>Resolved prior Staff field persistence mismatch</t>
         </is>
       </c>
     </row>
@@ -4052,27 +4020,27 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Supplier/Credit</t>
+          <t>Shopping</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Architecture Split</t>
+          <t>Product Catalog</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Supplier purchases and customer credits</t>
+          <t>Product-only shopping screen</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>SK-W2-007</t>
+          <t>SK-W2-010</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Split old credit module into supplier-purchases and customer-credits APIs/services; updated supplier route to /supplier</t>
+          <t>Separated Shopping product catalog from Orders flow and disabled native invalid styling with noValidate</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -4082,17 +4050,17 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>No Change</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>No Change</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>No Change</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -4102,22 +4070,22 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>90</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -4127,7 +4095,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>Manual old route regression pending</t>
+          <t>Orders now handled by dedicated Orders page</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -4142,7 +4110,7 @@
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>Old Credit.jsx/Credit.css and creditRoutes removed</t>
+          <t>Cleaner module ownership</t>
         </is>
       </c>
     </row>
@@ -4169,82 +4137,82 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Customers</t>
+          <t>All</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Customer Product Entries</t>
+          <t>Build Verification</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Edit/delete product entry support</t>
+          <t>Frontend production build</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>SK-W2-008</t>
+          <t>SK-QA-002</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Added customer product entry update/delete service and route support</t>
+          <t>Ran frontend production build after latest Staff and Shopping updates</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
+          <t>No Change</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>No Change</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>No Change</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>Build Passed</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>65</t>
-        </is>
-      </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>Need confirm UI exposes edit/delete actions</t>
+          <t>None</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -4254,19 +4222,19 @@
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>Backend/service ready</t>
+          <t>vite build passed with 117 modules</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -4286,52 +4254,52 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Transactions</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Build Verification</t>
+          <t>Unified Ledger</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Frontend production build</t>
+          <t>Transactions page/API</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>SK-QA-001</t>
+          <t>SK-W2-003</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Ran frontend production build after Staff/Orders/Supplier changes</t>
+          <t>Implement active Transactions route/page and backend unified transaction API</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>No Change</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>No Change</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>No Change</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Passed</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -4341,49 +4309,49 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>8</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>0</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>To Do</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Route not active in sidebar/app</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>vite build passed with 117 modules</t>
+          <t>Still placeholder file only</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -4403,27 +4371,27 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Transactions</t>
+          <t>Reports</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Unified Ledger</t>
+          <t>Reports</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Transactions page/API</t>
+          <t>Business reports</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>SK-W2-003</t>
+          <t>SK-W2-004</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Implement active Transactions route/page and backend unified transaction API</t>
+          <t>Build Reports page with filters and export-ready summaries</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -4478,261 +4446,27 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>Route not active in sidebar/app</t>
+          <t>Depends report data contract</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>Still placeholder file only</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Adesh/Dev Team</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>SmartKhata</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Sprint 2</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Reports</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Reports</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Business reports</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>SK-W2-004</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>Build Reports page with filters and export-ready summaries</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="S13" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-      <c r="T13" t="inlineStr">
-        <is>
-          <t>Depends report data contract</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>2026-07-03</t>
-        </is>
-      </c>
-      <c r="V13" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
-      <c r="W13" t="inlineStr">
-        <is>
           <t>Still placeholder</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Adesh/Dev Team</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>SmartKhata</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Sprint 2</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Settings</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Settings</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>App settings</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>SK-008</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>Create settings page for shop/profile/security/config</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="S14" t="inlineStr">
-        <is>
-          <t>To Do</t>
-        </is>
-      </c>
-      <c r="T14" t="inlineStr">
-        <is>
-          <t>Scope not finalized</t>
-        </is>
-      </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>2026-07-04</t>
-        </is>
-      </c>
-      <c r="V14" t="inlineStr">
-        <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="W14" t="inlineStr">
-        <is>
-          <t>Still placeholder</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:W14"/>
+  <autoFilter ref="A1:W12"/>
 </worksheet>
 </file>
 
@@ -4794,22 +4528,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SK-W2-006</t>
+          <t>SK-W2-009</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>01 Jul: Complete Staff CRUD verification and fix form/backend mismatches</t>
+          <t>01 Jul: QA Staff HRMS expansion and attendance save/history flow</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>02 Jul: Add attendance/salary/advance UI panels</t>
+          <t>02 Jul: Connect salary/advance UI to existing backend APIs</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>03 Jul: QA staff history and summary totals</t>
+          <t>03 Jul: Replace static staff report/document data with real data or clear placeholders</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -4829,34 +4563,34 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>QA</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SK-W2-008</t>
+          <t>SK-W2-010</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>01 Jul: Verify customer product entry edit/delete service and route</t>
+          <t>01 Jul: Verify Shopping product-only catalog after Orders split</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>02 Jul: Add edit/delete controls in Customers UI if missing</t>
+          <t>02 Jul: Regression test Orders page</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>03 Jul: Regression test customer balances</t>
+          <t>03 Jul: Confirm dashboard order/product data remains accurate</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -4866,12 +4600,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Customer product entry API</t>
+          <t>Shopping and Orders APIs</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>QA</t>
         </is>
       </c>
     </row>
@@ -4962,12 +4696,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SK-QA-002</t>
+          <t>SK-QA-003</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>01 Jul: Run frontend build and smoke checklist</t>
+          <t>01 Jul: Run frontend build and update project Excel</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -5133,7 +4867,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>78</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -5195,7 +4929,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>45</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -5279,17 +5013,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Staff and credit architecture</t>
+          <t>Staff HRMS and shopping ownership cleanup</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Staff/Supplier/Customer Credits</t>
+          <t>Staff/Shopping</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Staff + credit split</t>
+          <t>Staff management and product catalog</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -5304,12 +5038,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Staff API and split credit APIs</t>
+          <t>Staff API and shopping product API</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -5319,17 +5053,17 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>88</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>QA</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Staff core CRUD added; supplier/customer credit APIs split</t>
+          <t>Staff field persistence fixed; attendance UI added; Shopping separated from Orders</t>
         </is>
       </c>
     </row>
@@ -5552,7 +5286,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -5567,7 +5301,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -5799,7 +5533,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -5809,7 +5543,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>48%</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -5826,24 +5560,24 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Orders implementation, Staff module, supplier/customer credit split, transactions/reports next</t>
+          <t>Orders implementation, Staff HRMS expansion, supplier/customer credit split, transactions/reports next</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>Known open bugs tracked</t>
@@ -5856,7 +5590,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>55%</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -5903,7 +5637,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>10%</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -5950,7 +5684,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>10%</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -6315,7 +6049,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>88</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -6335,7 +6069,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>22</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -6350,7 +6084,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>82</t>
         </is>
       </c>
     </row>
@@ -6409,42 +6143,42 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>88</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
           <t>86</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>80</t>
-        </is>
-      </c>
       <c r="E10" t="inlineStr">
         <is>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
           <t>86</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>78</t>
         </is>
       </c>
     </row>
@@ -6968,7 +6702,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Product catalog, product CRUD, filters, preview modal</t>
+          <t>Product catalog, product CRUD, filters, preview modal, Google/direct image URL normalization</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -6983,7 +6717,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>88</t>
         </is>
       </c>
     </row>
@@ -7059,12 +6793,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Staff Management</t>
+          <t>Staff HRMS</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Staff summary, add/edit/delete form, searchable staff list, staff profile</t>
+          <t>Staff dashboard, registration, filters, profile, attendance entry/history, salary/advance/leave/performance/document/report sections</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -7074,12 +6808,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>QA</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>88</t>
         </is>
       </c>
     </row>
@@ -7606,7 +7340,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Staff CRUD, summary, attendance, salary payments, advance payments, history</t>
+          <t>Staff CRUD, persisted staff_id/email/department, summary, attendance, salary payments, advance payments, history</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -7621,12 +7355,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>QA</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>86</t>
+          <t>90</t>
         </is>
       </c>
     </row>
@@ -8112,7 +7846,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Staff profile records</t>
+          <t>Staff profile records including staff_id/email/department</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -8132,7 +7866,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>88</t>
         </is>
       </c>
     </row>
@@ -8164,7 +7898,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>78</t>
         </is>
       </c>
     </row>
@@ -8196,7 +7930,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>72</t>
         </is>
       </c>
     </row>
@@ -8228,7 +7962,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>72</t>
         </is>
       </c>
     </row>

</xml_diff>